<commit_message>
updated prj with parallel testing, cross browser testing, reports, implemented data driven and log4j
updated prj with parallel testing, cross browser testing, reports, implemented data driven and log4j
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData/Excel_Login_Pythoncode.xlsx
+++ b/src/test/resources/TestData/Excel_Login_Pythoncode.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\geeta\eclipse-workspace-2023\GitDesktop\DsAlgo_Scrutinizers_Prj\src\test\resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16416497-F3C7-46FB-A6D2-BF2C4BE5D3D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7AD6F62-D08F-4188-BCBC-704EECE6842C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14685" yWindow="3000" windowWidth="14115" windowHeight="13095" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2640" yWindow="2640" windowWidth="21600" windowHeight="12645" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LogIn" sheetId="1" r:id="rId1"/>
     <sheet name="pythonCode" sheetId="2" r:id="rId2"/>
+    <sheet name="Valid LogIn" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="26">
   <si>
     <t>username</t>
   </si>
@@ -1505,7 +1506,7 @@
   <dimension ref="A1:B1000"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="168.85546875" customWidth="1"/>
+    <col min="1" max="1" width="122.140625" customWidth="1"/>
     <col min="2" max="2" width="48.5703125" customWidth="1"/>
     <col min="3" max="6" width="14.42578125" customWidth="1"/>
   </cols>
@@ -2582,4 +2583,41 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55F14B74-135A-4E89-8AC8-C49289628EAF}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>